<commit_message>
Fix QUDT namespace bug in augment_w_definitions.ipynb; regenerate definitions
</commit_message>
<xml_diff>
--- a/projects/project-3/assignment/src/data/ccom-qudt-structural-matches-with-defs.xlsx
+++ b/projects/project-3/assignment/src/data/ccom-qudt-structural-matches-with-defs.xlsx
@@ -610,7 +610,11 @@
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -698,7 +702,11 @@
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -830,7 +838,11 @@
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1050,7 +1062,11 @@
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1270,7 +1286,11 @@
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1358,7 +1378,11 @@
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1490,7 +1514,11 @@
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1710,7 +1738,11 @@
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1930,7 +1962,11 @@
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2018,7 +2054,11 @@
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2150,7 +2190,11 @@
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2370,7 +2414,11 @@
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2590,7 +2638,11 @@
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2678,7 +2730,11 @@
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2810,7 +2866,11 @@
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3030,7 +3090,11 @@
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3250,7 +3314,11 @@
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3338,7 +3406,11 @@
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3470,7 +3542,11 @@
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3690,7 +3766,11 @@
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3910,7 +3990,11 @@
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3998,7 +4082,11 @@
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4130,7 +4218,11 @@
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4350,7 +4442,11 @@
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4570,7 +4666,11 @@
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4658,7 +4758,11 @@
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4790,7 +4894,11 @@
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5010,7 +5118,11 @@
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5230,7 +5342,11 @@
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5318,7 +5434,11 @@
         </is>
       </c>
       <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5450,7 +5570,11 @@
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5670,7 +5794,11 @@
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5890,7 +6018,11 @@
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5978,7 +6110,11 @@
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6110,7 +6246,11 @@
         </is>
       </c>
       <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6330,7 +6470,11 @@
         </is>
       </c>
       <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6550,7 +6694,11 @@
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
-      <c r="J139" t="inlineStr"/>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6638,7 +6786,11 @@
         </is>
       </c>
       <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6770,7 +6922,11 @@
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6990,7 +7146,11 @@
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7210,7 +7370,11 @@
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7298,7 +7462,11 @@
         </is>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7430,7 +7598,11 @@
         </is>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" t="inlineStr"/>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7650,7 +7822,11 @@
         </is>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7870,7 +8046,11 @@
         </is>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7958,7 +8138,11 @@
         </is>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8090,7 +8274,11 @@
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" t="inlineStr"/>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8310,7 +8498,11 @@
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" t="inlineStr"/>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8530,7 +8722,11 @@
         </is>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" t="inlineStr"/>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8618,7 +8814,11 @@
         </is>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" t="inlineStr"/>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -8750,7 +8950,11 @@
         </is>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" t="inlineStr"/>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8970,7 +9174,11 @@
         </is>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9190,7 +9398,11 @@
         </is>
       </c>
       <c r="I199" t="inlineStr"/>
-      <c r="J199" t="inlineStr"/>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9278,7 +9490,11 @@
         </is>
       </c>
       <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr"/>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9410,7 +9626,11 @@
         </is>
       </c>
       <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -9630,7 +9850,11 @@
         </is>
       </c>
       <c r="I209" t="inlineStr"/>
-      <c r="J209" t="inlineStr"/>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -9850,7 +10074,11 @@
         </is>
       </c>
       <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr"/>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -9938,7 +10166,11 @@
         </is>
       </c>
       <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -10070,7 +10302,11 @@
         </is>
       </c>
       <c r="I219" t="inlineStr"/>
-      <c r="J219" t="inlineStr"/>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -10290,7 +10526,11 @@
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
-      <c r="J224" t="inlineStr"/>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -10510,7 +10750,11 @@
         </is>
       </c>
       <c r="I229" t="inlineStr"/>
-      <c r="J229" t="inlineStr"/>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -10598,7 +10842,11 @@
         </is>
       </c>
       <c r="I231" t="inlineStr"/>
-      <c r="J231" t="inlineStr"/>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -10730,7 +10978,11 @@
         </is>
       </c>
       <c r="I234" t="inlineStr"/>
-      <c r="J234" t="inlineStr"/>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -10950,7 +11202,11 @@
         </is>
       </c>
       <c r="I239" t="inlineStr"/>
-      <c r="J239" t="inlineStr"/>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -11170,7 +11426,11 @@
         </is>
       </c>
       <c r="I244" t="inlineStr"/>
-      <c r="J244" t="inlineStr"/>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -11258,7 +11518,11 @@
         </is>
       </c>
       <c r="I246" t="inlineStr"/>
-      <c r="J246" t="inlineStr"/>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -11390,7 +11654,11 @@
         </is>
       </c>
       <c r="I249" t="inlineStr"/>
-      <c r="J249" t="inlineStr"/>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -11610,7 +11878,11 @@
         </is>
       </c>
       <c r="I254" t="inlineStr"/>
-      <c r="J254" t="inlineStr"/>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -11830,7 +12102,11 @@
         </is>
       </c>
       <c r="I259" t="inlineStr"/>
-      <c r="J259" t="inlineStr"/>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -11918,7 +12194,11 @@
         </is>
       </c>
       <c r="I261" t="inlineStr"/>
-      <c r="J261" t="inlineStr"/>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -12050,7 +12330,11 @@
         </is>
       </c>
       <c r="I264" t="inlineStr"/>
-      <c r="J264" t="inlineStr"/>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -12270,7 +12554,11 @@
         </is>
       </c>
       <c r="I269" t="inlineStr"/>
-      <c r="J269" t="inlineStr"/>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -12490,7 +12778,11 @@
         </is>
       </c>
       <c r="I274" t="inlineStr"/>
-      <c r="J274" t="inlineStr"/>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -12578,7 +12870,11 @@
         </is>
       </c>
       <c r="I276" t="inlineStr"/>
-      <c r="J276" t="inlineStr"/>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -12710,7 +13006,11 @@
         </is>
       </c>
       <c r="I279" t="inlineStr"/>
-      <c r="J279" t="inlineStr"/>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -12930,7 +13230,11 @@
         </is>
       </c>
       <c r="I284" t="inlineStr"/>
-      <c r="J284" t="inlineStr"/>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -13150,7 +13454,11 @@
         </is>
       </c>
       <c r="I289" t="inlineStr"/>
-      <c r="J289" t="inlineStr"/>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -13238,7 +13546,11 @@
         </is>
       </c>
       <c r="I291" t="inlineStr"/>
-      <c r="J291" t="inlineStr"/>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -13370,7 +13682,11 @@
         </is>
       </c>
       <c r="I294" t="inlineStr"/>
-      <c r="J294" t="inlineStr"/>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -13590,7 +13906,11 @@
         </is>
       </c>
       <c r="I299" t="inlineStr"/>
-      <c r="J299" t="inlineStr"/>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -13810,7 +14130,11 @@
         </is>
       </c>
       <c r="I304" t="inlineStr"/>
-      <c r="J304" t="inlineStr"/>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -13898,7 +14222,11 @@
         </is>
       </c>
       <c r="I306" t="inlineStr"/>
-      <c r="J306" t="inlineStr"/>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -14030,7 +14358,11 @@
         </is>
       </c>
       <c r="I309" t="inlineStr"/>
-      <c r="J309" t="inlineStr"/>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -14250,7 +14582,11 @@
         </is>
       </c>
       <c r="I314" t="inlineStr"/>
-      <c r="J314" t="inlineStr"/>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -14470,7 +14806,11 @@
         </is>
       </c>
       <c r="I319" t="inlineStr"/>
-      <c r="J319" t="inlineStr"/>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -14558,7 +14898,11 @@
         </is>
       </c>
       <c r="I321" t="inlineStr"/>
-      <c r="J321" t="inlineStr"/>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -14690,7 +15034,11 @@
         </is>
       </c>
       <c r="I324" t="inlineStr"/>
-      <c r="J324" t="inlineStr"/>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -14910,7 +15258,11 @@
         </is>
       </c>
       <c r="I329" t="inlineStr"/>
-      <c r="J329" t="inlineStr"/>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -15130,7 +15482,11 @@
         </is>
       </c>
       <c r="I334" t="inlineStr"/>
-      <c r="J334" t="inlineStr"/>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -15218,7 +15574,11 @@
         </is>
       </c>
       <c r="I336" t="inlineStr"/>
-      <c r="J336" t="inlineStr"/>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -15350,7 +15710,11 @@
         </is>
       </c>
       <c r="I339" t="inlineStr"/>
-      <c r="J339" t="inlineStr"/>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -15570,7 +15934,11 @@
         </is>
       </c>
       <c r="I344" t="inlineStr"/>
-      <c r="J344" t="inlineStr"/>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -15790,7 +16158,11 @@
         </is>
       </c>
       <c r="I349" t="inlineStr"/>
-      <c r="J349" t="inlineStr"/>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -15878,7 +16250,11 @@
         </is>
       </c>
       <c r="I351" t="inlineStr"/>
-      <c r="J351" t="inlineStr"/>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -16010,7 +16386,11 @@
         </is>
       </c>
       <c r="I354" t="inlineStr"/>
-      <c r="J354" t="inlineStr"/>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -16230,7 +16610,11 @@
         </is>
       </c>
       <c r="I359" t="inlineStr"/>
-      <c r="J359" t="inlineStr"/>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -16450,7 +16834,11 @@
         </is>
       </c>
       <c r="I364" t="inlineStr"/>
-      <c r="J364" t="inlineStr"/>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -16538,7 +16926,11 @@
         </is>
       </c>
       <c r="I366" t="inlineStr"/>
-      <c r="J366" t="inlineStr"/>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -16670,7 +17062,11 @@
         </is>
       </c>
       <c r="I369" t="inlineStr"/>
-      <c r="J369" t="inlineStr"/>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -16890,7 +17286,11 @@
         </is>
       </c>
       <c r="I374" t="inlineStr"/>
-      <c r="J374" t="inlineStr"/>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -17110,7 +17510,11 @@
         </is>
       </c>
       <c r="I379" t="inlineStr"/>
-      <c r="J379" t="inlineStr"/>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -17198,7 +17602,11 @@
         </is>
       </c>
       <c r="I381" t="inlineStr"/>
-      <c r="J381" t="inlineStr"/>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -17330,7 +17738,11 @@
         </is>
       </c>
       <c r="I384" t="inlineStr"/>
-      <c r="J384" t="inlineStr"/>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -17550,7 +17962,11 @@
         </is>
       </c>
       <c r="I389" t="inlineStr"/>
-      <c r="J389" t="inlineStr"/>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -17770,7 +18186,11 @@
         </is>
       </c>
       <c r="I394" t="inlineStr"/>
-      <c r="J394" t="inlineStr"/>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -17858,7 +18278,11 @@
         </is>
       </c>
       <c r="I396" t="inlineStr"/>
-      <c r="J396" t="inlineStr"/>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -17990,7 +18414,11 @@
         </is>
       </c>
       <c r="I399" t="inlineStr"/>
-      <c r="J399" t="inlineStr"/>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -18210,7 +18638,11 @@
         </is>
       </c>
       <c r="I404" t="inlineStr"/>
-      <c r="J404" t="inlineStr"/>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -18430,7 +18862,11 @@
         </is>
       </c>
       <c r="I409" t="inlineStr"/>
-      <c r="J409" t="inlineStr"/>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -18518,7 +18954,11 @@
         </is>
       </c>
       <c r="I411" t="inlineStr"/>
-      <c r="J411" t="inlineStr"/>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -18650,7 +19090,11 @@
         </is>
       </c>
       <c r="I414" t="inlineStr"/>
-      <c r="J414" t="inlineStr"/>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -18870,7 +19314,11 @@
         </is>
       </c>
       <c r="I419" t="inlineStr"/>
-      <c r="J419" t="inlineStr"/>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -19090,7 +19538,11 @@
         </is>
       </c>
       <c r="I424" t="inlineStr"/>
-      <c r="J424" t="inlineStr"/>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -19178,7 +19630,11 @@
         </is>
       </c>
       <c r="I426" t="inlineStr"/>
-      <c r="J426" t="inlineStr"/>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -19310,7 +19766,11 @@
         </is>
       </c>
       <c r="I429" t="inlineStr"/>
-      <c r="J429" t="inlineStr"/>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -19530,7 +19990,11 @@
         </is>
       </c>
       <c r="I434" t="inlineStr"/>
-      <c r="J434" t="inlineStr"/>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -19750,7 +20214,11 @@
         </is>
       </c>
       <c r="I439" t="inlineStr"/>
-      <c r="J439" t="inlineStr"/>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -19838,7 +20306,11 @@
         </is>
       </c>
       <c r="I441" t="inlineStr"/>
-      <c r="J441" t="inlineStr"/>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -19970,7 +20442,11 @@
         </is>
       </c>
       <c r="I444" t="inlineStr"/>
-      <c r="J444" t="inlineStr"/>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -20190,7 +20666,11 @@
         </is>
       </c>
       <c r="I449" t="inlineStr"/>
-      <c r="J449" t="inlineStr"/>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -20410,7 +20890,11 @@
         </is>
       </c>
       <c r="I454" t="inlineStr"/>
-      <c r="J454" t="inlineStr"/>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -20498,7 +20982,11 @@
         </is>
       </c>
       <c r="I456" t="inlineStr"/>
-      <c r="J456" t="inlineStr"/>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -20630,7 +21118,11 @@
         </is>
       </c>
       <c r="I459" t="inlineStr"/>
-      <c r="J459" t="inlineStr"/>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -20850,7 +21342,11 @@
         </is>
       </c>
       <c r="I464" t="inlineStr"/>
-      <c r="J464" t="inlineStr"/>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -21070,7 +21566,11 @@
         </is>
       </c>
       <c r="I469" t="inlineStr"/>
-      <c r="J469" t="inlineStr"/>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -21158,7 +21658,11 @@
         </is>
       </c>
       <c r="I471" t="inlineStr"/>
-      <c r="J471" t="inlineStr"/>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -21290,7 +21794,11 @@
         </is>
       </c>
       <c r="I474" t="inlineStr"/>
-      <c r="J474" t="inlineStr"/>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -21510,7 +22018,11 @@
         </is>
       </c>
       <c r="I479" t="inlineStr"/>
-      <c r="J479" t="inlineStr"/>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -21730,7 +22242,11 @@
         </is>
       </c>
       <c r="I484" t="inlineStr"/>
-      <c r="J484" t="inlineStr"/>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -21818,7 +22334,11 @@
         </is>
       </c>
       <c r="I486" t="inlineStr"/>
-      <c r="J486" t="inlineStr"/>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -21950,7 +22470,11 @@
         </is>
       </c>
       <c r="I489" t="inlineStr"/>
-      <c r="J489" t="inlineStr"/>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -22170,7 +22694,11 @@
         </is>
       </c>
       <c r="I494" t="inlineStr"/>
-      <c r="J494" t="inlineStr"/>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -22390,7 +22918,11 @@
         </is>
       </c>
       <c r="I499" t="inlineStr"/>
-      <c r="J499" t="inlineStr"/>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -22478,7 +23010,11 @@
         </is>
       </c>
       <c r="I501" t="inlineStr"/>
-      <c r="J501" t="inlineStr"/>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -22610,7 +23146,11 @@
         </is>
       </c>
       <c r="I504" t="inlineStr"/>
-      <c r="J504" t="inlineStr"/>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
@@ -22830,7 +23370,11 @@
         </is>
       </c>
       <c r="I509" t="inlineStr"/>
-      <c r="J509" t="inlineStr"/>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -23050,7 +23594,11 @@
         </is>
       </c>
       <c r="I514" t="inlineStr"/>
-      <c r="J514" t="inlineStr"/>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -23138,7 +23686,11 @@
         </is>
       </c>
       <c r="I516" t="inlineStr"/>
-      <c r="J516" t="inlineStr"/>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
@@ -23270,7 +23822,11 @@
         </is>
       </c>
       <c r="I519" t="inlineStr"/>
-      <c r="J519" t="inlineStr"/>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -23490,7 +24046,11 @@
         </is>
       </c>
       <c r="I524" t="inlineStr"/>
-      <c r="J524" t="inlineStr"/>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
@@ -23710,7 +24270,11 @@
         </is>
       </c>
       <c r="I529" t="inlineStr"/>
-      <c r="J529" t="inlineStr"/>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -23798,7 +24362,11 @@
         </is>
       </c>
       <c r="I531" t="inlineStr"/>
-      <c r="J531" t="inlineStr"/>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -23930,7 +24498,11 @@
         </is>
       </c>
       <c r="I534" t="inlineStr"/>
-      <c r="J534" t="inlineStr"/>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -24150,7 +24722,11 @@
         </is>
       </c>
       <c r="I539" t="inlineStr"/>
-      <c r="J539" t="inlineStr"/>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -24370,7 +24946,11 @@
         </is>
       </c>
       <c r="I544" t="inlineStr"/>
-      <c r="J544" t="inlineStr"/>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -24458,7 +25038,11 @@
         </is>
       </c>
       <c r="I546" t="inlineStr"/>
-      <c r="J546" t="inlineStr"/>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -24590,7 +25174,11 @@
         </is>
       </c>
       <c r="I549" t="inlineStr"/>
-      <c r="J549" t="inlineStr"/>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -24810,7 +25398,11 @@
         </is>
       </c>
       <c r="I554" t="inlineStr"/>
-      <c r="J554" t="inlineStr"/>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="555">
       <c r="A555" t="inlineStr">
@@ -25030,7 +25622,11 @@
         </is>
       </c>
       <c r="I559" t="inlineStr"/>
-      <c r="J559" t="inlineStr"/>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
@@ -25118,7 +25714,11 @@
         </is>
       </c>
       <c r="I561" t="inlineStr"/>
-      <c r="J561" t="inlineStr"/>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
@@ -25250,7 +25850,11 @@
         </is>
       </c>
       <c r="I564" t="inlineStr"/>
-      <c r="J564" t="inlineStr"/>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -25470,7 +26074,11 @@
         </is>
       </c>
       <c r="I569" t="inlineStr"/>
-      <c r="J569" t="inlineStr"/>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
@@ -25690,7 +26298,11 @@
         </is>
       </c>
       <c r="I574" t="inlineStr"/>
-      <c r="J574" t="inlineStr"/>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
@@ -25778,7 +26390,11 @@
         </is>
       </c>
       <c r="I576" t="inlineStr"/>
-      <c r="J576" t="inlineStr"/>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
@@ -25910,7 +26526,11 @@
         </is>
       </c>
       <c r="I579" t="inlineStr"/>
-      <c r="J579" t="inlineStr"/>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
@@ -26130,7 +26750,11 @@
         </is>
       </c>
       <c r="I584" t="inlineStr"/>
-      <c r="J584" t="inlineStr"/>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -26350,7 +26974,11 @@
         </is>
       </c>
       <c r="I589" t="inlineStr"/>
-      <c r="J589" t="inlineStr"/>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
@@ -26438,7 +27066,11 @@
         </is>
       </c>
       <c r="I591" t="inlineStr"/>
-      <c r="J591" t="inlineStr"/>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -26570,7 +27202,11 @@
         </is>
       </c>
       <c r="I594" t="inlineStr"/>
-      <c r="J594" t="inlineStr"/>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
@@ -26790,7 +27426,11 @@
         </is>
       </c>
       <c r="I599" t="inlineStr"/>
-      <c r="J599" t="inlineStr"/>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
@@ -27010,7 +27650,11 @@
         </is>
       </c>
       <c r="I604" t="inlineStr"/>
-      <c r="J604" t="inlineStr"/>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -27098,7 +27742,11 @@
         </is>
       </c>
       <c r="I606" t="inlineStr"/>
-      <c r="J606" t="inlineStr"/>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
@@ -27230,7 +27878,11 @@
         </is>
       </c>
       <c r="I609" t="inlineStr"/>
-      <c r="J609" t="inlineStr"/>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
@@ -27450,7 +28102,11 @@
         </is>
       </c>
       <c r="I614" t="inlineStr"/>
-      <c r="J614" t="inlineStr"/>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
@@ -27670,7 +28326,11 @@
         </is>
       </c>
       <c r="I619" t="inlineStr"/>
-      <c r="J619" t="inlineStr"/>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -27758,7 +28418,11 @@
         </is>
       </c>
       <c r="I621" t="inlineStr"/>
-      <c r="J621" t="inlineStr"/>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
@@ -27890,7 +28554,11 @@
         </is>
       </c>
       <c r="I624" t="inlineStr"/>
-      <c r="J624" t="inlineStr"/>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
@@ -28110,7 +28778,11 @@
         </is>
       </c>
       <c r="I629" t="inlineStr"/>
-      <c r="J629" t="inlineStr"/>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
@@ -28330,7 +29002,11 @@
         </is>
       </c>
       <c r="I634" t="inlineStr"/>
-      <c r="J634" t="inlineStr"/>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>Thermodynamics units are units that provide reference scales for quantifying the conversion of energy into work, as well as heat and its relation to macroscopic variables such as temperature and pressure.</t>
+        </is>
+      </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -28418,7 +29094,11 @@
         </is>
       </c>
       <c r="I636" t="inlineStr"/>
-      <c r="J636" t="inlineStr"/>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>This class contains units that measure financial quantities, such as currency, transactions, rates of return, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -28550,7 +29230,11 @@
         </is>
       </c>
       <c r="I639" t="inlineStr"/>
-      <c r="J639" t="inlineStr"/>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>units for measuring human resources</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
@@ -28770,7 +29454,11 @@
         </is>
       </c>
       <c r="I644" t="inlineStr"/>
-      <c r="J644" t="inlineStr"/>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>The class of units used to measure the properties of electricity and magnetism.</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">

</xml_diff>